<commit_message>
output 폴더(balcony, bed, diffuser) 데이터 추가
</commit_message>
<xml_diff>
--- a/output_balcony/balcony_100_products.xlsx
+++ b/output_balcony/balcony_100_products.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -540,12 +540,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>라이트그레이</t>
+          <t>그레이</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -564,15 +564,9 @@
       <c r="N2" t="n">
         <v>18000</v>
       </c>
-      <c r="O2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="b">
-        <v>0</v>
-      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -616,7 +610,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -626,7 +620,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -635,15 +629,9 @@
       <c r="N3" t="n">
         <v>20610</v>
       </c>
-      <c r="O3" t="b">
-        <v>0</v>
-      </c>
-      <c r="P3" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="b">
-        <v>0</v>
-      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -682,12 +670,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>라이트 브라운</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -697,7 +685,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -706,15 +694,9 @@
       <c r="N4" t="n">
         <v>26910</v>
       </c>
-      <c r="O4" t="b">
-        <v>0</v>
-      </c>
-      <c r="P4" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="b">
-        <v>0</v>
-      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -753,12 +735,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>다크그레이</t>
+          <t>그레이</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -768,7 +750,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -777,15 +759,9 @@
       <c r="N5" t="n">
         <v>20610</v>
       </c>
-      <c r="O5" t="b">
-        <v>0</v>
-      </c>
-      <c r="P5" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="b">
-        <v>0</v>
-      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -824,12 +800,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>다크그레이</t>
+          <t>그레이</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -839,7 +815,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -848,15 +824,9 @@
       <c r="N6" t="n">
         <v>44910</v>
       </c>
-      <c r="O6" t="b">
-        <v>0</v>
-      </c>
-      <c r="P6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="b">
-        <v>0</v>
-      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -895,12 +865,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>라이트 브라운</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -910,7 +880,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -919,15 +889,9 @@
       <c r="N7" t="n">
         <v>27000</v>
       </c>
-      <c r="O7" t="b">
-        <v>0</v>
-      </c>
-      <c r="P7" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="b">
-        <v>0</v>
-      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -966,12 +930,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>라이트 브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -981,7 +945,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -990,15 +954,9 @@
       <c r="N8" t="n">
         <v>206010</v>
       </c>
-      <c r="O8" t="b">
-        <v>0</v>
-      </c>
-      <c r="P8" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="b">
-        <v>0</v>
-      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1042,7 +1000,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1052,7 +1010,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1061,15 +1019,9 @@
       <c r="N9" t="n">
         <v>80010</v>
       </c>
-      <c r="O9" t="b">
-        <v>0</v>
-      </c>
-      <c r="P9" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="b">
-        <v>0</v>
-      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1113,7 +1065,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1123,7 +1075,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1132,15 +1084,9 @@
       <c r="N10" t="n">
         <v>80010</v>
       </c>
-      <c r="O10" t="b">
-        <v>0</v>
-      </c>
-      <c r="P10" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="b">
-        <v>0</v>
-      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1179,12 +1125,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>다크블루</t>
+          <t>블루</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1194,7 +1140,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -1203,15 +1149,9 @@
       <c r="N11" t="n">
         <v>80910</v>
       </c>
-      <c r="O11" t="b">
-        <v>0</v>
-      </c>
-      <c r="P11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="b">
-        <v>0</v>
-      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1250,12 +1190,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>오프화이트</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1265,7 +1205,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -1274,15 +1214,9 @@
       <c r="N12" t="n">
         <v>80910</v>
       </c>
-      <c r="O12" t="b">
-        <v>0</v>
-      </c>
-      <c r="P12" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="b">
-        <v>0</v>
-      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1321,12 +1255,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>앤트러싸이트</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1336,7 +1270,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1345,15 +1279,9 @@
       <c r="N13" t="n">
         <v>80910</v>
       </c>
-      <c r="O13" t="b">
-        <v>0</v>
-      </c>
-      <c r="P13" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="b">
-        <v>0</v>
-      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1397,7 +1325,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1407,7 +1335,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1416,15 +1344,9 @@
       <c r="N14" t="n">
         <v>430920</v>
       </c>
-      <c r="O14" t="b">
-        <v>0</v>
-      </c>
-      <c r="P14" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="b">
-        <v>0</v>
-      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1463,12 +1385,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>아연도금</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1478,7 +1400,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1487,15 +1409,9 @@
       <c r="N15" t="n">
         <v>430920</v>
       </c>
-      <c r="O15" t="b">
-        <v>0</v>
-      </c>
-      <c r="P15" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="b">
-        <v>0</v>
-      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1539,7 +1455,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1549,7 +1465,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1558,15 +1474,9 @@
       <c r="N16" t="n">
         <v>139320</v>
       </c>
-      <c r="O16" t="b">
-        <v>0</v>
-      </c>
-      <c r="P16" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="b">
-        <v>0</v>
-      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1610,7 +1520,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1620,7 +1530,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1629,15 +1539,9 @@
       <c r="N17" t="n">
         <v>139320</v>
       </c>
-      <c r="O17" t="b">
-        <v>0</v>
-      </c>
-      <c r="P17" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="b">
-        <v>0</v>
-      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1681,7 +1585,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1691,7 +1595,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1700,15 +1604,9 @@
       <c r="N18" t="n">
         <v>89910</v>
       </c>
-      <c r="O18" t="b">
-        <v>0</v>
-      </c>
-      <c r="P18" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="b">
-        <v>0</v>
-      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1752,7 +1650,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1762,7 +1660,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1771,15 +1669,9 @@
       <c r="N19" t="n">
         <v>152010</v>
       </c>
-      <c r="O19" t="b">
-        <v>0</v>
-      </c>
-      <c r="P19" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q19" t="b">
-        <v>0</v>
-      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1823,7 +1715,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1833,7 +1725,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1842,15 +1734,9 @@
       <c r="N20" t="n">
         <v>143820</v>
       </c>
-      <c r="O20" t="b">
-        <v>0</v>
-      </c>
-      <c r="P20" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="b">
-        <v>0</v>
-      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1894,7 +1780,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1904,7 +1790,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -1913,15 +1799,9 @@
       <c r="N21" t="n">
         <v>89910</v>
       </c>
-      <c r="O21" t="b">
-        <v>0</v>
-      </c>
-      <c r="P21" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q21" t="b">
-        <v>0</v>
-      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1965,7 +1845,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1975,7 +1855,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -1984,15 +1864,9 @@
       <c r="N22" t="n">
         <v>53910</v>
       </c>
-      <c r="O22" t="b">
-        <v>0</v>
-      </c>
-      <c r="P22" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q22" t="b">
-        <v>0</v>
-      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2036,7 +1910,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2046,7 +1920,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2055,15 +1929,9 @@
       <c r="N23" t="n">
         <v>90810</v>
       </c>
-      <c r="O23" t="b">
-        <v>0</v>
-      </c>
-      <c r="P23" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q23" t="b">
-        <v>0</v>
-      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2107,7 +1975,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2117,7 +1985,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -2126,15 +1994,9 @@
       <c r="N24" t="n">
         <v>90810</v>
       </c>
-      <c r="O24" t="b">
-        <v>0</v>
-      </c>
-      <c r="P24" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="b">
-        <v>0</v>
-      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2178,7 +2040,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2188,7 +2050,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -2197,15 +2059,9 @@
       <c r="N25" t="n">
         <v>50310</v>
       </c>
-      <c r="O25" t="b">
-        <v>0</v>
-      </c>
-      <c r="P25" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q25" t="b">
-        <v>0</v>
-      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2249,7 +2105,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2259,7 +2115,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -2268,15 +2124,9 @@
       <c r="N26" t="n">
         <v>50310</v>
       </c>
-      <c r="O26" t="b">
-        <v>0</v>
-      </c>
-      <c r="P26" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q26" t="b">
-        <v>0</v>
-      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2320,7 +2170,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2330,7 +2180,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -2339,15 +2189,9 @@
       <c r="N27" t="n">
         <v>112320</v>
       </c>
-      <c r="O27" t="b">
-        <v>0</v>
-      </c>
-      <c r="P27" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q27" t="b">
-        <v>0</v>
-      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2391,7 +2235,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2401,7 +2245,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -2410,15 +2254,9 @@
       <c r="N28" t="n">
         <v>112320</v>
       </c>
-      <c r="O28" t="b">
-        <v>0</v>
-      </c>
-      <c r="P28" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q28" t="b">
-        <v>0</v>
-      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2462,7 +2300,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2472,7 +2310,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -2481,15 +2319,9 @@
       <c r="N29" t="n">
         <v>145620</v>
       </c>
-      <c r="O29" t="b">
-        <v>0</v>
-      </c>
-      <c r="P29" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q29" t="b">
-        <v>0</v>
-      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2533,7 +2365,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2543,7 +2375,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -2552,15 +2384,9 @@
       <c r="N30" t="n">
         <v>53910</v>
       </c>
-      <c r="O30" t="b">
-        <v>0</v>
-      </c>
-      <c r="P30" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="b">
-        <v>0</v>
-      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2599,12 +2425,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>라이트 브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2614,7 +2440,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -2623,15 +2449,9 @@
       <c r="N31" t="n">
         <v>134100</v>
       </c>
-      <c r="O31" t="b">
-        <v>0</v>
-      </c>
-      <c r="P31" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q31" t="b">
-        <v>0</v>
-      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2670,12 +2490,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>접이식 다크브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2685,7 +2505,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -2694,15 +2514,9 @@
       <c r="N32" t="n">
         <v>277740</v>
       </c>
-      <c r="O32" t="b">
-        <v>0</v>
-      </c>
-      <c r="P32" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q32" t="b">
-        <v>0</v>
-      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2741,12 +2555,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>접이식 다크브라운 프뢰쇤 두브홀멘 베이지</t>
+          <t>베이지</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2756,7 +2570,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -2765,15 +2579,9 @@
       <c r="N33" t="n">
         <v>331380</v>
       </c>
-      <c r="O33" t="b">
-        <v>0</v>
-      </c>
-      <c r="P33" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q33" t="b">
-        <v>0</v>
-      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2808,12 +2616,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>접이식 다크브라운 쿠다르나 라이트그레이베이지</t>
+          <t>베이지</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2823,7 +2631,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2832,15 +2640,9 @@
       <c r="N34" t="n">
         <v>306180</v>
       </c>
-      <c r="O34" t="b">
-        <v>0</v>
-      </c>
-      <c r="P34" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q34" t="b">
-        <v>0</v>
-      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2875,12 +2677,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>접이식 다크브라운 클뢰산 다크블루</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2890,7 +2692,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2899,15 +2701,9 @@
       <c r="N35" t="n">
         <v>306180</v>
       </c>
-      <c r="O35" t="b">
-        <v>0</v>
-      </c>
-      <c r="P35" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q35" t="b">
-        <v>0</v>
-      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2946,7 +2742,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>라이트 브라운</t>
+          <t>그린</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2970,15 +2766,9 @@
       <c r="N36" t="n">
         <v>44910</v>
       </c>
-      <c r="O36" t="b">
-        <v>0</v>
-      </c>
-      <c r="P36" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q36" t="b">
-        <v>0</v>
-      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3017,7 +2807,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>다크그린</t>
+          <t>그린</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3041,15 +2831,9 @@
       <c r="N37" t="n">
         <v>17910</v>
       </c>
-      <c r="O37" t="b">
-        <v>0</v>
-      </c>
-      <c r="P37" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q37" t="b">
-        <v>0</v>
-      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3093,7 +2877,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3103,7 +2887,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -3112,15 +2896,9 @@
       <c r="N38" t="n">
         <v>9000</v>
       </c>
-      <c r="O38" t="b">
-        <v>0</v>
-      </c>
-      <c r="P38" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q38" t="b">
-        <v>0</v>
-      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3159,12 +2937,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>라이트 브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3174,7 +2952,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -3183,15 +2961,9 @@
       <c r="N39" t="n">
         <v>58410</v>
       </c>
-      <c r="O39" t="b">
-        <v>0</v>
-      </c>
-      <c r="P39" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q39" t="b">
-        <v>0</v>
-      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3230,12 +3002,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>다크브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3245,7 +3017,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -3254,15 +3026,9 @@
       <c r="N40" t="n">
         <v>112230</v>
       </c>
-      <c r="O40" t="b">
-        <v>0</v>
-      </c>
-      <c r="P40" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q40" t="b">
-        <v>0</v>
-      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3301,12 +3067,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>다크브라운 프뢰쇤 두브홀멘 베이지</t>
+          <t>베이지</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3316,7 +3082,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -3325,15 +3091,9 @@
       <c r="N41" t="n">
         <v>139050</v>
       </c>
-      <c r="O41" t="b">
-        <v>0</v>
-      </c>
-      <c r="P41" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q41" t="b">
-        <v>0</v>
-      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3368,12 +3128,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>다크브라운 쿠다르나 라이트그레이베이지</t>
+          <t>베이지</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3383,7 +3143,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3392,15 +3152,9 @@
       <c r="N42" t="n">
         <v>126450</v>
       </c>
-      <c r="O42" t="b">
-        <v>0</v>
-      </c>
-      <c r="P42" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q42" t="b">
-        <v>0</v>
-      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3435,12 +3189,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>접이식 다크브라운 클뢰산 다크블루</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3450,7 +3204,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3459,15 +3213,9 @@
       <c r="N43" t="n">
         <v>126450</v>
       </c>
-      <c r="O43" t="b">
-        <v>0</v>
-      </c>
-      <c r="P43" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q43" t="b">
-        <v>0</v>
-      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3506,7 +3254,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>라이트그린</t>
+          <t>그린</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -3530,15 +3278,9 @@
       <c r="N44" t="n">
         <v>18000</v>
       </c>
-      <c r="O44" t="b">
-        <v>0</v>
-      </c>
-      <c r="P44" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q44" t="b">
-        <v>0</v>
-      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3582,7 +3324,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3592,7 +3334,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3601,15 +3343,9 @@
       <c r="N45" t="n">
         <v>18000</v>
       </c>
-      <c r="O45" t="b">
-        <v>0</v>
-      </c>
-      <c r="P45" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q45" t="b">
-        <v>0</v>
-      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3648,12 +3384,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>옐로</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3663,7 +3399,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3672,15 +3408,9 @@
       <c r="N46" t="n">
         <v>18000</v>
       </c>
-      <c r="O46" t="b">
-        <v>0</v>
-      </c>
-      <c r="P46" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q46" t="b">
-        <v>0</v>
-      </c>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3724,7 +3454,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3734,7 +3464,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3743,15 +3473,9 @@
       <c r="N47" t="n">
         <v>18000</v>
       </c>
-      <c r="O47" t="b">
-        <v>0</v>
-      </c>
-      <c r="P47" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q47" t="b">
-        <v>0</v>
-      </c>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3790,7 +3514,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>태양열 스트라이프 라이트그린</t>
+          <t>그린</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -3814,15 +3538,9 @@
       <c r="N48" t="n">
         <v>15210</v>
       </c>
-      <c r="O48" t="b">
-        <v>0</v>
-      </c>
-      <c r="P48" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q48" t="b">
-        <v>0</v>
-      </c>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3861,12 +3579,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>브라이트레드</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3876,7 +3594,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M49" t="n">
@@ -3885,15 +3603,9 @@
       <c r="N49" t="n">
         <v>62910</v>
       </c>
-      <c r="O49" t="b">
-        <v>0</v>
-      </c>
-      <c r="P49" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q49" t="b">
-        <v>0</v>
-      </c>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3932,12 +3644,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>오프화이트</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3947,7 +3659,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M50" t="n">
@@ -3956,15 +3668,9 @@
       <c r="N50" t="n">
         <v>62910</v>
       </c>
-      <c r="O50" t="b">
-        <v>0</v>
-      </c>
-      <c r="P50" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q50" t="b">
-        <v>0</v>
-      </c>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4003,12 +3709,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>앤트러싸이트</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -4018,7 +3724,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M51" t="n">
@@ -4027,15 +3733,9 @@
       <c r="N51" t="n">
         <v>62910</v>
       </c>
-      <c r="O51" t="b">
-        <v>0</v>
-      </c>
-      <c r="P51" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q51" t="b">
-        <v>0</v>
-      </c>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4074,12 +3774,12 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>다크블루</t>
+          <t>블루</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -4089,7 +3789,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="M52" t="n">
@@ -4098,15 +3798,9 @@
       <c r="N52" t="n">
         <v>62910</v>
       </c>
-      <c r="O52" t="b">
-        <v>0</v>
-      </c>
-      <c r="P52" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q52" t="b">
-        <v>0</v>
-      </c>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4145,12 +3839,12 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>라이트 브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4160,7 +3854,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M53" t="n">
@@ -4169,15 +3863,9 @@
       <c r="N53" t="n">
         <v>35910</v>
       </c>
-      <c r="O53" t="b">
-        <v>0</v>
-      </c>
-      <c r="P53" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q53" t="b">
-        <v>0</v>
-      </c>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4216,12 +3904,12 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>라이트 브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -4231,7 +3919,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M54" t="n">
@@ -4240,15 +3928,9 @@
       <c r="N54" t="n">
         <v>80910</v>
       </c>
-      <c r="O54" t="b">
-        <v>0</v>
-      </c>
-      <c r="P54" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q54" t="b">
-        <v>0</v>
-      </c>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4287,12 +3969,12 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>블랙 리스</t>
+          <t>블랙</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -4302,7 +3984,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M55" t="n">
@@ -4311,15 +3993,9 @@
       <c r="N55" t="n">
         <v>180000</v>
       </c>
-      <c r="O55" t="b">
-        <v>0</v>
-      </c>
-      <c r="P55" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q55" t="b">
-        <v>0</v>
-      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4358,12 +4034,12 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>접이식 라이트 브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4373,7 +4049,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M56" t="n">
@@ -4382,15 +4058,9 @@
       <c r="N56" t="n">
         <v>25110</v>
       </c>
-      <c r="O56" t="b">
-        <v>0</v>
-      </c>
-      <c r="P56" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q56" t="b">
-        <v>0</v>
-      </c>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4429,12 +4099,12 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>다크옐로</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4444,7 +4114,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M57" t="n">
@@ -4453,15 +4123,9 @@
       <c r="N57" t="n">
         <v>8910</v>
       </c>
-      <c r="O57" t="b">
-        <v>0</v>
-      </c>
-      <c r="P57" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q57" t="b">
-        <v>0</v>
-      </c>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4500,12 +4164,12 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>파도 모양 태양열 혼합 색상</t>
+          <t>화이트</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4515,7 +4179,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M58" t="n">
@@ -4524,15 +4188,9 @@
       <c r="N58" t="n">
         <v>8910</v>
       </c>
-      <c r="O58" t="b">
-        <v>0</v>
-      </c>
-      <c r="P58" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q58" t="b">
-        <v>0</v>
-      </c>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4576,7 +4234,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4586,7 +4244,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M59" t="n">
@@ -4595,15 +4253,9 @@
       <c r="N59" t="n">
         <v>34110</v>
       </c>
-      <c r="O59" t="b">
-        <v>0</v>
-      </c>
-      <c r="P59" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q59" t="b">
-        <v>0</v>
-      </c>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4642,12 +4294,12 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>라이트 브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4657,7 +4309,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M60" t="n">
@@ -4666,15 +4318,9 @@
       <c r="N60" t="n">
         <v>62910</v>
       </c>
-      <c r="O60" t="b">
-        <v>0</v>
-      </c>
-      <c r="P60" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q60" t="b">
-        <v>0</v>
-      </c>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4718,7 +4364,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4728,7 +4374,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>etc</t>
         </is>
       </c>
       <c r="M61" t="n">
@@ -4737,15 +4383,9 @@
       <c r="N61" t="n">
         <v>35910</v>
       </c>
-      <c r="O61" t="b">
-        <v>0</v>
-      </c>
-      <c r="P61" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q61" t="b">
-        <v>0</v>
-      </c>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4784,12 +4424,12 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>블랙 라이트 브라운</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4799,7 +4439,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M62" t="n">
@@ -4808,15 +4448,9 @@
       <c r="N62" t="n">
         <v>77130</v>
       </c>
-      <c r="O62" t="b">
-        <v>0</v>
-      </c>
-      <c r="P62" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q62" t="b">
-        <v>0</v>
-      </c>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4855,12 +4489,12 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>블랙 라이트브라운 프뢰쇤 두브홀멘 베이지</t>
+          <t>베이지</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4870,7 +4504,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M63" t="n">
@@ -4879,15 +4513,9 @@
       <c r="N63" t="n">
         <v>103950</v>
       </c>
-      <c r="O63" t="b">
-        <v>0</v>
-      </c>
-      <c r="P63" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q63" t="b">
-        <v>0</v>
-      </c>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4922,12 +4550,12 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>블랙 라이트브라운 접이식 접이식 KUDDARNA 쿠다르나 라이트그레이베이지</t>
+          <t>베이지</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4937,7 +4565,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M64" t="n">
@@ -4946,15 +4574,9 @@
       <c r="N64" t="n">
         <v>91350</v>
       </c>
-      <c r="O64" t="b">
-        <v>0</v>
-      </c>
-      <c r="P64" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q64" t="b">
-        <v>0</v>
-      </c>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4989,12 +4611,12 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>접이식 블랙 라이트브라운 접이식 KLÖSAN 클뢰산 다크블루</t>
+          <t>우드</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -5004,7 +4626,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>autumn</t>
         </is>
       </c>
       <c r="M65" t="n">
@@ -5013,15 +4635,9 @@
       <c r="N65" t="n">
         <v>91350</v>
       </c>
-      <c r="O65" t="b">
-        <v>0</v>
-      </c>
-      <c r="P65" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q65" t="b">
-        <v>0</v>
-      </c>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5060,12 +4676,12 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>다크그레이</t>
+          <t>그레이</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -5075,7 +4691,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M66" t="n">
@@ -5084,15 +4700,9 @@
       <c r="N66" t="n">
         <v>4500</v>
       </c>
-      <c r="O66" t="b">
-        <v>0</v>
-      </c>
-      <c r="P66" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q66" t="b">
-        <v>0</v>
-      </c>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5131,12 +4741,12 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>다크그레이</t>
+          <t>그레이</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -5146,7 +4756,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>spring</t>
+          <t>winter</t>
         </is>
       </c>
       <c r="M67" t="n">
@@ -5155,15 +4765,9 @@
       <c r="N67" t="n">
         <v>2700</v>
       </c>
-      <c r="O67" t="b">
-        <v>0</v>
-      </c>
-      <c r="P67" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q67" t="b">
-        <v>0</v>
-      </c>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>